<commit_message>
added custom functions tests for type hints
</commit_message>
<xml_diff>
--- a/xlwingsjs/tests/udf_tests_officejs.xlsx
+++ b/xlwingsjs/tests/udf_tests_officejs.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10211"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10714"/>
   <workbookPr showInkAnnotation="0" codeName="ThisWorkbook" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/felix/dev/xlwings/xlwingsjs/tests/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB61C120-ACDD-C44C-BB7D-B2A9432C88F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64F41CCA-4CF8-6140-967D-54A3A4EFCE84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-1860" yWindow="-21100" windowWidth="38400" windowHeight="21100" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -130,7 +130,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="285" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="130">
   <si>
     <t>epected</t>
   </si>
@@ -505,6 +505,21 @@
   </si>
   <si>
     <t>varargs_arg_decorator</t>
+  </si>
+  <si>
+    <t>type_hints_arg</t>
+  </si>
+  <si>
+    <t>type_hints_arg_annotated</t>
+  </si>
+  <si>
+    <t>type_hints_ret_annotated</t>
+  </si>
+  <si>
+    <t>type_hints_ret_decorator_override</t>
+  </si>
+  <si>
+    <t>type_hints_arg_decorator_coexistence</t>
   </si>
 </sst>
 </file>
@@ -664,7 +679,14 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="4">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -1225,6 +1247,12 @@
         <we:customFunctionIds>_xldudf_XLWINGSJS_READ_VERTICAL_NPARRAY</we:customFunctionIds>
         <we:customFunctionIds>_xldudf_XLWINGSJS_READ_WORKBOOK_CALLER</we:customFunctionIds>
         <we:customFunctionIds>_xldudf_XLWINGSJS_RETURN_PD_NAT</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_XLWINGSJS_TYPE_HINTS_ARG</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_XLWINGSJS_TYPE_HINTS_ARG_ANNOTATED</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_XLWINGSJS_TYPE_HINTS_ARG_DECORATOR_COEXISTENCE</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_XLWINGSJS_TYPE_HINTS_RET_ANNOTATED</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_XLWINGSJS_TYPE_HINTS_RET_DECORATOR_OVERRIDE</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_XLWINGSJS_VARARGS_ARG_DECORATOR</we:customFunctionIds>
         <we:customFunctionIds>_xldudf_XLWINGSJS_VARIABLE_ARGS</we:customFunctionIds>
         <we:customFunctionIds>_xldudf_XLWINGSJS_VOLATILE</we:customFunctionIds>
         <we:customFunctionIds>_xldudf_XLWINGSJS_WRITE_2DLIST</we:customFunctionIds>
@@ -1272,7 +1300,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:P358"/>
+  <dimension ref="A1:P378"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="39" bestFit="1" customWidth="1"/>
@@ -7349,19 +7377,285 @@
         <v>1</v>
       </c>
     </row>
+    <row r="360" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A360" t="b">
+        <f>G360</f>
+        <v>1</v>
+      </c>
+      <c r="B360" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="E360" t="s">
+        <v>110</v>
+      </c>
+      <c r="F360" t="s">
+        <v>111</v>
+      </c>
+      <c r="G360" s="2" t="b" cm="1">
+        <f t="array" ref="G360">_xldudf_XLWINGSJS_TYPE_HINTS_ARG(D360:F362)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="361" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="D361">
+        <v>0</v>
+      </c>
+      <c r="E361">
+        <v>1</v>
+      </c>
+      <c r="F361">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="362" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="D362">
+        <v>1</v>
+      </c>
+      <c r="E362">
+        <v>3</v>
+      </c>
+      <c r="F362">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="364" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A364" t="b">
+        <f>G364</f>
+        <v>1</v>
+      </c>
+      <c r="B364" s="23" t="s">
+        <v>126</v>
+      </c>
+      <c r="E364" t="s">
+        <v>110</v>
+      </c>
+      <c r="F364" t="s">
+        <v>111</v>
+      </c>
+      <c r="G364" s="2" t="b" cm="1">
+        <f t="array" ref="G364">_xldudf_XLWINGSJS_TYPE_HINTS_ARG_ANNOTATED(D364:F366)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="365" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="D365">
+        <v>0</v>
+      </c>
+      <c r="E365">
+        <v>1</v>
+      </c>
+      <c r="F365">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="366" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="D366">
+        <v>1</v>
+      </c>
+      <c r="E366">
+        <v>3</v>
+      </c>
+      <c r="F366">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="368" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A368" t="b">
+        <f>AND(_xlfn.ANCHORARRAY(J368))</f>
+        <v>1</v>
+      </c>
+      <c r="B368" s="23" t="s">
+        <v>127</v>
+      </c>
+      <c r="E368" t="s">
+        <v>110</v>
+      </c>
+      <c r="F368" t="s">
+        <v>111</v>
+      </c>
+      <c r="G368" s="2" t="str" cm="1">
+        <f t="array" ref="G368:H370">_xldudf_XLWINGSJS_TYPE_HINTS_RET_ANNOTATED()</f>
+        <v>one</v>
+      </c>
+      <c r="H368" s="2" t="str">
+        <v>two</v>
+      </c>
+      <c r="J368" t="b" cm="1">
+        <f t="array" ref="J368:K370">_xlfn.ANCHORARRAY(G368)=E368:F370</f>
+        <v>1</v>
+      </c>
+      <c r="K368" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="369" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="E369">
+        <v>1</v>
+      </c>
+      <c r="F369">
+        <v>2</v>
+      </c>
+      <c r="G369" s="2">
+        <v>1</v>
+      </c>
+      <c r="H369" s="2">
+        <v>2</v>
+      </c>
+      <c r="J369" t="b">
+        <v>1</v>
+      </c>
+      <c r="K369" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="370" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="E370">
+        <v>3</v>
+      </c>
+      <c r="F370">
+        <v>4</v>
+      </c>
+      <c r="G370" s="2">
+        <v>3</v>
+      </c>
+      <c r="H370" s="2">
+        <v>4</v>
+      </c>
+      <c r="J370" t="b">
+        <v>1</v>
+      </c>
+      <c r="K370" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="372" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A372" t="b">
+        <f>AND(_xlfn.ANCHORARRAY(J372))</f>
+        <v>1</v>
+      </c>
+      <c r="B372" s="23" t="s">
+        <v>128</v>
+      </c>
+      <c r="E372" t="s">
+        <v>110</v>
+      </c>
+      <c r="F372" t="s">
+        <v>111</v>
+      </c>
+      <c r="G372" s="2" t="str" cm="1">
+        <f t="array" ref="G372:H374">_xldudf_XLWINGSJS_TYPE_HINTS_RET_DECORATOR_OVERRIDE()</f>
+        <v>one</v>
+      </c>
+      <c r="H372" s="2" t="str">
+        <v>two</v>
+      </c>
+      <c r="J372" t="b" cm="1">
+        <f t="array" ref="J372:K374">_xlfn.ANCHORARRAY(G372)=E372:F374</f>
+        <v>1</v>
+      </c>
+      <c r="K372" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="373" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="E373">
+        <v>1</v>
+      </c>
+      <c r="F373">
+        <v>2</v>
+      </c>
+      <c r="G373" s="2">
+        <v>1</v>
+      </c>
+      <c r="H373" s="2">
+        <v>2</v>
+      </c>
+      <c r="J373" t="b">
+        <v>1</v>
+      </c>
+      <c r="K373" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="374" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="E374">
+        <v>3</v>
+      </c>
+      <c r="F374">
+        <v>4</v>
+      </c>
+      <c r="G374" s="2">
+        <v>3</v>
+      </c>
+      <c r="H374" s="2">
+        <v>4</v>
+      </c>
+      <c r="J374" t="b">
+        <v>1</v>
+      </c>
+      <c r="K374" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="376" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A376" t="b">
+        <f>G376</f>
+        <v>1</v>
+      </c>
+      <c r="B376" s="23" t="s">
+        <v>129</v>
+      </c>
+      <c r="E376" t="s">
+        <v>110</v>
+      </c>
+      <c r="F376" t="s">
+        <v>111</v>
+      </c>
+      <c r="G376" s="2" t="b" cm="1">
+        <f t="array" ref="G376">_xldudf_XLWINGSJS_TYPE_HINTS_ARG_DECORATOR_COEXISTENCE(D376:F378)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="377" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="D377">
+        <v>0</v>
+      </c>
+      <c r="E377">
+        <v>1</v>
+      </c>
+      <c r="F377">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="378" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="D378">
+        <v>1</v>
+      </c>
+      <c r="E378">
+        <v>3</v>
+      </c>
+      <c r="F378">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="A3:A97 A99:A170 A172:A283 A285 A289:A290 A298 A302 A306 A309 A312:A313 A317 A319:A1048576">
-    <cfRule type="containsErrors" dxfId="2" priority="18">
+  <conditionalFormatting sqref="A3:A97 A99:A170 A172:A283 A285 A289:A290 A298 A302 A306 A309 A312:A313 A317 A319:A359 A379:A1048576">
+    <cfRule type="containsErrors" dxfId="3" priority="19">
       <formula>ISERROR(A3)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A3:A170 A172:A1048576">
-    <cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="FALSE">
+  <conditionalFormatting sqref="A3:A170">
+    <cfRule type="containsText" dxfId="2" priority="2" operator="containsText" text="FALSE">
       <formula>NOT(ISERROR(SEARCH("FALSE",A3)))</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="A172:A1048576">
+    <cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="FALSE">
+      <formula>NOT(ISERROR(SEARCH("FALSE",A172)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="B3">
-    <cfRule type="cellIs" dxfId="0" priority="17" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="0" priority="18" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
more type hint tests
</commit_message>
<xml_diff>
--- a/xlwingsjs/tests/udf_tests_officejs.xlsx
+++ b/xlwingsjs/tests/udf_tests_officejs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/felix/dev/xlwings/xlwingsjs/tests/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64F41CCA-4CF8-6140-967D-54A3A4EFCE84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1CB7C6D-979D-6544-9794-A4693865A94F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-1860" yWindow="-21100" windowWidth="38400" windowHeight="21100" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -130,7 +130,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="313" uniqueCount="141">
   <si>
     <t>epected</t>
   </si>
@@ -507,19 +507,52 @@
     <t>varargs_arg_decorator</t>
   </si>
   <si>
-    <t>type_hints_arg</t>
-  </si>
-  <si>
-    <t>type_hints_arg_annotated</t>
-  </si>
-  <si>
-    <t>type_hints_ret_annotated</t>
-  </si>
-  <si>
-    <t>type_hints_ret_decorator_override</t>
-  </si>
-  <si>
-    <t>type_hints_arg_decorator_coexistence</t>
+    <t>type_hints_arg_float</t>
+  </si>
+  <si>
+    <t>type_hints_arg_str</t>
+  </si>
+  <si>
+    <t>type_hints_arg_bool</t>
+  </si>
+  <si>
+    <t>type_hints_arg_int</t>
+  </si>
+  <si>
+    <t>type_hints_arg_datetime</t>
+  </si>
+  <si>
+    <t>type_hints_arg_df</t>
+  </si>
+  <si>
+    <t>type_hints_arg_df_annotated</t>
+  </si>
+  <si>
+    <t>type_hints_ret_df_annotated</t>
+  </si>
+  <si>
+    <t>type_hints_ret_df_decorator_override</t>
+  </si>
+  <si>
+    <t>type_hints_arg_df_decorator_coexistence</t>
+  </si>
+  <si>
+    <t>type_hints_arg_list</t>
+  </si>
+  <si>
+    <t>type_hints_arg_list_int</t>
+  </si>
+  <si>
+    <t>type_hints_arg_list_list_int</t>
+  </si>
+  <si>
+    <t>type_hints_arg_dict</t>
+  </si>
+  <si>
+    <t>type_hints_arg_array</t>
+  </si>
+  <si>
+    <t>type_hints_arg_ndarray</t>
   </si>
 </sst>
 </file>
@@ -529,7 +562,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="m/d/yyyy\ h:mm:ss"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -581,8 +614,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -607,6 +647,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC5D9F1"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -621,7 +667,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -674,6 +720,11 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1166,7 +1217,7 @@
 
 <file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
 <wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
-  <wetp:taskpane dockstate="right" visibility="0" width="0" row="0">
+  <wetp:taskpane dockstate="right" visibility="0" width="350" row="0">
     <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </wetp:taskpane>
 </wetp:taskpanes>
@@ -1247,11 +1298,22 @@
         <we:customFunctionIds>_xldudf_XLWINGSJS_READ_VERTICAL_NPARRAY</we:customFunctionIds>
         <we:customFunctionIds>_xldudf_XLWINGSJS_READ_WORKBOOK_CALLER</we:customFunctionIds>
         <we:customFunctionIds>_xldudf_XLWINGSJS_RETURN_PD_NAT</we:customFunctionIds>
-        <we:customFunctionIds>_xldudf_XLWINGSJS_TYPE_HINTS_ARG</we:customFunctionIds>
-        <we:customFunctionIds>_xldudf_XLWINGSJS_TYPE_HINTS_ARG_ANNOTATED</we:customFunctionIds>
-        <we:customFunctionIds>_xldudf_XLWINGSJS_TYPE_HINTS_ARG_DECORATOR_COEXISTENCE</we:customFunctionIds>
-        <we:customFunctionIds>_xldudf_XLWINGSJS_TYPE_HINTS_RET_ANNOTATED</we:customFunctionIds>
-        <we:customFunctionIds>_xldudf_XLWINGSJS_TYPE_HINTS_RET_DECORATOR_OVERRIDE</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_XLWINGSJS_TYPE_HINTS_ARG_ARRAY</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_XLWINGSJS_TYPE_HINTS_ARG_BOOL</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_XLWINGSJS_TYPE_HINTS_ARG_DATETIME</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_XLWINGSJS_TYPE_HINTS_ARG_DF</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_XLWINGSJS_TYPE_HINTS_ARG_DF_ANNOTATED</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_XLWINGSJS_TYPE_HINTS_ARG_DF_DECORATOR_COEXISTENCE</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_XLWINGSJS_TYPE_HINTS_ARG_DICT</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_XLWINGSJS_TYPE_HINTS_ARG_FLOAT</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_XLWINGSJS_TYPE_HINTS_ARG_INT</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_XLWINGSJS_TYPE_HINTS_ARG_LIST</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_XLWINGSJS_TYPE_HINTS_ARG_LIST_INT</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_XLWINGSJS_TYPE_HINTS_ARG_LIST_LIST_INT</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_XLWINGSJS_TYPE_HINTS_ARG_NDARRAY</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_XLWINGSJS_TYPE_HINTS_ARG_STR</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_XLWINGSJS_TYPE_HINTS_RET_DF_ANNOTATED</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_XLWINGSJS_TYPE_HINTS_RET_DF_DECORATOR_OVERRIDE</we:customFunctionIds>
         <we:customFunctionIds>_xldudf_XLWINGSJS_VARARGS_ARG_DECORATOR</we:customFunctionIds>
         <we:customFunctionIds>_xldudf_XLWINGSJS_VARIABLE_ARGS</we:customFunctionIds>
         <we:customFunctionIds>_xldudf_XLWINGSJS_VOLATILE</we:customFunctionIds>
@@ -1300,7 +1362,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:P378"/>
+  <dimension ref="A1:P404"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="39" bestFit="1" customWidth="1"/>
@@ -7231,7 +7293,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="353" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="353" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A353" t="b">
         <f ca="1">G353</f>
         <v>1</v>
@@ -7244,7 +7306,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="355" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="355" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A355" t="b">
         <f>AND(K355:M358)</f>
         <v>1</v>
@@ -7281,7 +7343,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="356" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="356" spans="1:16" x14ac:dyDescent="0.2">
       <c r="D356">
         <v>0</v>
       </c>
@@ -7313,7 +7375,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="357" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="357" spans="1:16" x14ac:dyDescent="0.2">
       <c r="D357">
         <v>0</v>
       </c>
@@ -7345,7 +7407,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="358" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="358" spans="1:16" x14ac:dyDescent="0.2">
       <c r="D358">
         <v>0</v>
       </c>
@@ -7377,269 +7439,502 @@
         <v>1</v>
       </c>
     </row>
-    <row r="360" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A360" t="b">
-        <f>G360</f>
-        <v>1</v>
-      </c>
-      <c r="B360" s="23" t="s">
+    <row r="361" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A361" t="b">
+        <f>G361</f>
+        <v>1</v>
+      </c>
+      <c r="B361" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="C361" s="27"/>
+      <c r="D361" s="27"/>
+      <c r="E361" s="27"/>
+      <c r="F361" s="27">
+        <v>2</v>
+      </c>
+      <c r="G361" s="28" t="b" cm="1">
+        <f t="array" ref="G361">_xldudf_XLWINGSJS_TYPE_HINTS_ARG_INT(F361)</f>
+        <v>1</v>
+      </c>
+      <c r="H361" s="27"/>
+      <c r="I361" s="27"/>
+      <c r="J361" s="27"/>
+      <c r="K361" s="27"/>
+      <c r="L361" s="27"/>
+      <c r="M361" s="27"/>
+      <c r="N361" s="27"/>
+      <c r="O361" s="27"/>
+      <c r="P361" s="27"/>
+    </row>
+    <row r="363" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A363" t="b">
+        <f>G363</f>
+        <v>1</v>
+      </c>
+      <c r="B363" s="23" t="s">
         <v>125</v>
       </c>
-      <c r="E360" t="s">
+      <c r="F363">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="G363" s="2" t="b" cm="1">
+        <f t="array" ref="G363">_xldudf_XLWINGSJS_TYPE_HINTS_ARG_FLOAT(F363)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="365" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A365" t="b">
+        <f>G365</f>
+        <v>1</v>
+      </c>
+      <c r="B365" s="23" t="s">
+        <v>126</v>
+      </c>
+      <c r="F365" t="s">
+        <v>2</v>
+      </c>
+      <c r="G365" s="2" t="b" cm="1">
+        <f t="array" ref="G365">_xldudf_XLWINGSJS_TYPE_HINTS_ARG_STR(F365)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="367" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A367" t="b">
+        <f>G367</f>
+        <v>1</v>
+      </c>
+      <c r="B367" s="23" t="s">
+        <v>127</v>
+      </c>
+      <c r="F367" t="b">
+        <v>1</v>
+      </c>
+      <c r="G367" s="2" t="b" cm="1">
+        <f t="array" ref="G367">_xldudf_XLWINGSJS_TYPE_HINTS_ARG_BOOL(F367)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="368" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="B368" s="23"/>
+    </row>
+    <row r="369" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A369" t="b">
+        <f>G369</f>
+        <v>1</v>
+      </c>
+      <c r="B369" s="23" t="s">
+        <v>129</v>
+      </c>
+      <c r="F369" s="4">
+        <v>44185</v>
+      </c>
+      <c r="G369" s="2" t="b" cm="1">
+        <f t="array" ref="G369">_xldudf_XLWINGSJS_TYPE_HINTS_ARG_DATETIME(F369)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="371" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A371" t="b">
+        <f>G371</f>
+        <v>1</v>
+      </c>
+      <c r="B371" s="23" t="s">
+        <v>135</v>
+      </c>
+      <c r="E371">
+        <v>1</v>
+      </c>
+      <c r="F371">
+        <v>2</v>
+      </c>
+      <c r="G371" s="2" t="b" cm="1">
+        <f t="array" ref="G371">_xldudf_XLWINGSJS_TYPE_HINTS_ARG_LIST(E371:F371)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="373" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A373" t="b">
+        <f>G373</f>
+        <v>1</v>
+      </c>
+      <c r="B373" s="23" t="s">
+        <v>136</v>
+      </c>
+      <c r="E373">
+        <v>1</v>
+      </c>
+      <c r="F373">
+        <v>2</v>
+      </c>
+      <c r="G373" s="2" t="b" cm="1">
+        <f t="array" ref="G373">_xldudf_XLWINGSJS_TYPE_HINTS_ARG_LIST_INT(E373:F373)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="375" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A375" t="b">
+        <f>G375</f>
+        <v>1</v>
+      </c>
+      <c r="B375" s="23" t="s">
+        <v>137</v>
+      </c>
+      <c r="E375">
+        <v>1</v>
+      </c>
+      <c r="F375">
+        <v>2</v>
+      </c>
+      <c r="G375" s="2" t="b" cm="1">
+        <f t="array" ref="G375">_xldudf_XLWINGSJS_TYPE_HINTS_ARG_LIST_LIST_INT(E375:F376)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="376" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="E376">
+        <v>3</v>
+      </c>
+      <c r="F376">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="378" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A378" t="b">
+        <f>G378</f>
+        <v>1</v>
+      </c>
+      <c r="B378" s="23" t="s">
+        <v>138</v>
+      </c>
+      <c r="E378" t="s">
+        <v>50</v>
+      </c>
+      <c r="F378">
+        <v>1</v>
+      </c>
+      <c r="G378" s="2" t="b" cm="1">
+        <f t="array" ref="G378">_xldudf_XLWINGSJS_TYPE_HINTS_ARG_DICT(E378:F378)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="380" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A380" t="b">
+        <f>G380</f>
+        <v>1</v>
+      </c>
+      <c r="B380" s="23" t="s">
+        <v>139</v>
+      </c>
+      <c r="E380">
+        <v>1</v>
+      </c>
+      <c r="F380">
+        <v>2</v>
+      </c>
+      <c r="G380" s="2" t="b" cm="1">
+        <f t="array" ref="G380">_xldudf_XLWINGSJS_TYPE_HINTS_ARG_ARRAY(E380:F381)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="381" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="E381">
+        <v>3</v>
+      </c>
+      <c r="F381">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="383" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A383" t="b">
+        <f>G383</f>
+        <v>1</v>
+      </c>
+      <c r="B383" s="23" t="s">
+        <v>140</v>
+      </c>
+      <c r="E383">
+        <v>1</v>
+      </c>
+      <c r="F383">
+        <v>2</v>
+      </c>
+      <c r="G383" s="2" t="b" cm="1">
+        <f t="array" ref="G383">_xldudf_XLWINGSJS_TYPE_HINTS_ARG_NDARRAY(E383:F384)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="384" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="E384">
+        <v>3</v>
+      </c>
+      <c r="F384">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="386" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A386" t="b">
+        <f>G386</f>
+        <v>1</v>
+      </c>
+      <c r="B386" s="23" t="s">
+        <v>130</v>
+      </c>
+      <c r="E386" t="s">
         <v>110</v>
       </c>
-      <c r="F360" t="s">
+      <c r="F386" t="s">
         <v>111</v>
       </c>
-      <c r="G360" s="2" t="b" cm="1">
-        <f t="array" ref="G360">_xldudf_XLWINGSJS_TYPE_HINTS_ARG(D360:F362)</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="361" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="D361">
+      <c r="G386" s="2" t="b" cm="1">
+        <f t="array" ref="G386">_xldudf_XLWINGSJS_TYPE_HINTS_ARG_DF(D386:F388)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="387" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="D387">
         <v>0</v>
       </c>
-      <c r="E361">
-        <v>1</v>
-      </c>
-      <c r="F361">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="362" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="D362">
-        <v>1</v>
-      </c>
-      <c r="E362">
+      <c r="E387">
+        <v>1</v>
+      </c>
+      <c r="F387">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="388" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="D388">
+        <v>1</v>
+      </c>
+      <c r="E388">
         <v>3</v>
       </c>
-      <c r="F362">
+      <c r="F388">
         <v>4</v>
       </c>
     </row>
-    <row r="364" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A364" t="b">
-        <f>G364</f>
-        <v>1</v>
-      </c>
-      <c r="B364" s="23" t="s">
-        <v>126</v>
-      </c>
-      <c r="E364" t="s">
+    <row r="390" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A390" t="b">
+        <f>G390</f>
+        <v>1</v>
+      </c>
+      <c r="B390" s="23" t="s">
+        <v>131</v>
+      </c>
+      <c r="E390" t="s">
         <v>110</v>
       </c>
-      <c r="F364" t="s">
+      <c r="F390" t="s">
         <v>111</v>
       </c>
-      <c r="G364" s="2" t="b" cm="1">
-        <f t="array" ref="G364">_xldudf_XLWINGSJS_TYPE_HINTS_ARG_ANNOTATED(D364:F366)</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="365" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="D365">
+      <c r="G390" s="2" t="b" cm="1">
+        <f t="array" ref="G390">_xldudf_XLWINGSJS_TYPE_HINTS_ARG_DF_ANNOTATED(D390:F392)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="391" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="D391">
         <v>0</v>
       </c>
-      <c r="E365">
-        <v>1</v>
-      </c>
-      <c r="F365">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="366" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="D366">
-        <v>1</v>
-      </c>
-      <c r="E366">
+      <c r="E391">
+        <v>1</v>
+      </c>
+      <c r="F391">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="392" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="D392">
+        <v>1</v>
+      </c>
+      <c r="E392">
         <v>3</v>
       </c>
-      <c r="F366">
+      <c r="F392">
         <v>4</v>
       </c>
     </row>
-    <row r="368" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A368" t="b">
-        <f>AND(_xlfn.ANCHORARRAY(J368))</f>
-        <v>1</v>
-      </c>
-      <c r="B368" s="23" t="s">
-        <v>127</v>
-      </c>
-      <c r="E368" t="s">
+    <row r="394" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A394" t="b">
+        <f>AND(_xlfn.ANCHORARRAY(J394))</f>
+        <v>1</v>
+      </c>
+      <c r="B394" s="23" t="s">
+        <v>132</v>
+      </c>
+      <c r="E394" t="s">
         <v>110</v>
       </c>
-      <c r="F368" t="s">
+      <c r="F394" t="s">
         <v>111</v>
       </c>
-      <c r="G368" s="2" t="str" cm="1">
-        <f t="array" ref="G368:H370">_xldudf_XLWINGSJS_TYPE_HINTS_RET_ANNOTATED()</f>
+      <c r="G394" s="2" t="str" cm="1">
+        <f t="array" ref="G394:H396">_xldudf_XLWINGSJS_TYPE_HINTS_RET_DF_ANNOTATED()</f>
         <v>one</v>
       </c>
-      <c r="H368" s="2" t="str">
+      <c r="H394" s="2" t="str">
         <v>two</v>
       </c>
-      <c r="J368" t="b" cm="1">
-        <f t="array" ref="J368:K370">_xlfn.ANCHORARRAY(G368)=E368:F370</f>
-        <v>1</v>
-      </c>
-      <c r="K368" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="369" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E369">
-        <v>1</v>
-      </c>
-      <c r="F369">
-        <v>2</v>
-      </c>
-      <c r="G369" s="2">
-        <v>1</v>
-      </c>
-      <c r="H369" s="2">
-        <v>2</v>
-      </c>
-      <c r="J369" t="b">
-        <v>1</v>
-      </c>
-      <c r="K369" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="370" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E370">
+      <c r="J394" t="b" cm="1">
+        <f t="array" ref="J394:K396">_xlfn.ANCHORARRAY(G394)=E394:F396</f>
+        <v>1</v>
+      </c>
+      <c r="K394" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="395" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="E395">
+        <v>1</v>
+      </c>
+      <c r="F395">
+        <v>2</v>
+      </c>
+      <c r="G395" s="2">
+        <v>1</v>
+      </c>
+      <c r="H395" s="2">
+        <v>2</v>
+      </c>
+      <c r="J395" t="b">
+        <v>1</v>
+      </c>
+      <c r="K395" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="396" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="E396">
         <v>3</v>
       </c>
-      <c r="F370">
+      <c r="F396">
         <v>4</v>
       </c>
-      <c r="G370" s="2">
+      <c r="G396" s="2">
         <v>3</v>
       </c>
-      <c r="H370" s="2">
+      <c r="H396" s="2">
         <v>4</v>
       </c>
-      <c r="J370" t="b">
-        <v>1</v>
-      </c>
-      <c r="K370" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="372" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A372" t="b">
-        <f>AND(_xlfn.ANCHORARRAY(J372))</f>
-        <v>1</v>
-      </c>
-      <c r="B372" s="23" t="s">
-        <v>128</v>
-      </c>
-      <c r="E372" t="s">
+      <c r="J396" t="b">
+        <v>1</v>
+      </c>
+      <c r="K396" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="398" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A398" t="b">
+        <f>AND(_xlfn.ANCHORARRAY(J398))</f>
+        <v>1</v>
+      </c>
+      <c r="B398" s="23" t="s">
+        <v>133</v>
+      </c>
+      <c r="E398" t="s">
         <v>110</v>
       </c>
-      <c r="F372" t="s">
+      <c r="F398" t="s">
         <v>111</v>
       </c>
-      <c r="G372" s="2" t="str" cm="1">
-        <f t="array" ref="G372:H374">_xldudf_XLWINGSJS_TYPE_HINTS_RET_DECORATOR_OVERRIDE()</f>
+      <c r="G398" s="2" t="str" cm="1">
+        <f t="array" ref="G398:H400">_xldudf_XLWINGSJS_TYPE_HINTS_RET_DF_DECORATOR_OVERRIDE()</f>
         <v>one</v>
       </c>
-      <c r="H372" s="2" t="str">
+      <c r="H398" s="2" t="str">
         <v>two</v>
       </c>
-      <c r="J372" t="b" cm="1">
-        <f t="array" ref="J372:K374">_xlfn.ANCHORARRAY(G372)=E372:F374</f>
-        <v>1</v>
-      </c>
-      <c r="K372" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="373" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E373">
-        <v>1</v>
-      </c>
-      <c r="F373">
-        <v>2</v>
-      </c>
-      <c r="G373" s="2">
-        <v>1</v>
-      </c>
-      <c r="H373" s="2">
-        <v>2</v>
-      </c>
-      <c r="J373" t="b">
-        <v>1</v>
-      </c>
-      <c r="K373" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="374" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="E374">
+      <c r="J398" t="b" cm="1">
+        <f t="array" ref="J398:K400">_xlfn.ANCHORARRAY(G398)=E398:F400</f>
+        <v>1</v>
+      </c>
+      <c r="K398" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="399" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="E399">
+        <v>1</v>
+      </c>
+      <c r="F399">
+        <v>2</v>
+      </c>
+      <c r="G399" s="2">
+        <v>1</v>
+      </c>
+      <c r="H399" s="2">
+        <v>2</v>
+      </c>
+      <c r="J399" t="b">
+        <v>1</v>
+      </c>
+      <c r="K399" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="400" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="E400">
         <v>3</v>
       </c>
-      <c r="F374">
+      <c r="F400">
         <v>4</v>
       </c>
-      <c r="G374" s="2">
+      <c r="G400" s="2">
         <v>3</v>
       </c>
-      <c r="H374" s="2">
+      <c r="H400" s="2">
         <v>4</v>
       </c>
-      <c r="J374" t="b">
-        <v>1</v>
-      </c>
-      <c r="K374" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="376" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A376" t="b">
-        <f>G376</f>
-        <v>1</v>
-      </c>
-      <c r="B376" s="23" t="s">
-        <v>129</v>
-      </c>
-      <c r="E376" t="s">
+      <c r="J400" t="b">
+        <v>1</v>
+      </c>
+      <c r="K400" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="402" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A402" t="b">
+        <f>G402</f>
+        <v>1</v>
+      </c>
+      <c r="B402" s="23" t="s">
+        <v>134</v>
+      </c>
+      <c r="E402" t="s">
         <v>110</v>
       </c>
-      <c r="F376" t="s">
+      <c r="F402" t="s">
         <v>111</v>
       </c>
-      <c r="G376" s="2" t="b" cm="1">
-        <f t="array" ref="G376">_xldudf_XLWINGSJS_TYPE_HINTS_ARG_DECORATOR_COEXISTENCE(D376:F378)</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="377" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="D377">
+      <c r="G402" s="2" t="b" cm="1">
+        <f t="array" ref="G402">_xldudf_XLWINGSJS_TYPE_HINTS_ARG_DF_DECORATOR_COEXISTENCE(D402:F404)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="403" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="D403">
         <v>0</v>
       </c>
-      <c r="E377">
-        <v>1</v>
-      </c>
-      <c r="F377">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="378" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="D378">
-        <v>1</v>
-      </c>
-      <c r="E378">
+      <c r="E403">
+        <v>1</v>
+      </c>
+      <c r="F403">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="404" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="D404">
+        <v>1</v>
+      </c>
+      <c r="E404">
         <v>3</v>
       </c>
-      <c r="F378">
+      <c r="F404">
         <v>4</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A3:A97 A99:A170 A172:A283 A285 A289:A290 A298 A302 A306 A309 A312:A313 A317 A319:A359 A379:A1048576">
+  <conditionalFormatting sqref="A3:A97 A99:A170 A172:A283 A285 A289:A290 A298 A302 A306 A309 A312:A313 A317 A319:A360 A362 A366 A370 A405:A1048576 A372 A374 A376:A377 A379 A381:A382 A384:A385">
     <cfRule type="containsErrors" dxfId="3" priority="19">
       <formula>ISERROR(A3)</formula>
     </cfRule>

</xml_diff>